<commit_message>
Update V data - 2026-09-06 05:42:48
</commit_message>
<xml_diff>
--- a/data/V_data.xlsx
+++ b/data/V_data.xlsx
@@ -4717,7 +4717,7 @@
         <v>700273459200</v>
       </c>
       <c r="K2" t="n">
-        <v>32.250214</v>
+        <v>31.948042</v>
       </c>
       <c r="L2" t="n">
         <v>24.997501</v>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-09-06 05:35:02</t>
+          <t>2026-09-06 05:42:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update V data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/V_data.xlsx
+++ b/data/V_data.xlsx
@@ -4536,7 +4536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4657,25 +4657,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4723,7 +4743,7 @@
         <v>24.997501</v>
       </c>
       <c r="M2" t="n">
-        <v>11.63</v>
+        <v>11.74</v>
       </c>
       <c r="N2" t="n">
         <v>385.57</v>
@@ -4759,29 +4779,41 @@
       <c r="W2" t="n">
         <v>0.985</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>18.87</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>19.876524</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1704112694</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Credit Services</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://www.visa.com</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Visa Inc. operates as a payment technology company in the United States and internationally. The company operates VisaNet, a transaction processing network that enables authorization, clearing, and settlement of payment transactions. It also offers credit, debit, and prepaid card products; tap to pay, tokenization, and click to pay services; Visa Direct, a platform which facilitates money movement, enabling clients to collect, hold, convert, and send funds across its network; and issuing solutions, such as airport lounge access, dining reservations, shopping experiences, event tickets, and seller offers. In addition, the company provides acceptance solutions, an omnichannel payment integration with e-commerce platforms; risk detection and prevention solutions; and advisory and other services comprising consulting practice, proprietary analytics models, data scientists and economists, marketing services, and managed services. It provides its services under the Visa, Visa Electron, V PAY, Interlink, and PLUS brands. The company serves consumers, sellers, financial institutions, and government entities. Visa Inc. was founded in 1958 and is headquartered in San Francisco, California.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:42:03</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:10:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update V data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/V_data.xlsx
+++ b/data/V_data.xlsx
@@ -4757,15 +4757,11 @@
       <c r="Q2" t="n">
         <v>0.71</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.50782</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.66130996</v>
       </c>
       <c r="T2" t="n">
         <v>0.6119</v>
@@ -4813,7 +4809,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:49:10</t>
+          <t>2026-09-06 16:59:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update V data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/V_data.xlsx
+++ b/data/V_data.xlsx
@@ -4536,7 +4536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4677,25 +4677,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4787,29 +4802,38 @@
       <c r="AA2" t="n">
         <v>1704112694</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>44487999488</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>699948269568</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>31093999616</v>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Credit Services</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.visa.com</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Visa Inc. operates as a payment technology company in the United States and internationally. The company operates VisaNet, a transaction processing network that enables authorization, clearing, and settlement of payment transactions. It also offers credit, debit, and prepaid card products; tap to pay, tokenization, and click to pay services; Visa Direct, a platform which facilitates money movement, enabling clients to collect, hold, convert, and send funds across its network; and issuing solutions, such as airport lounge access, dining reservations, shopping experiences, event tickets, and seller offers. In addition, the company provides acceptance solutions, an omnichannel payment integration with e-commerce platforms; risk detection and prevention solutions; and advisory and other services comprising consulting practice, proprietary analytics models, data scientists and economists, marketing services, and managed services. It provides its services under the Visa, Visa Electron, V PAY, Interlink, and PLUS brands. The company serves consumers, sellers, financial institutions, and government entities. Visa Inc. was founded in 1958 and is headquartered in San Francisco, California.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:41</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:46</t>
         </is>
       </c>
     </row>

</xml_diff>